<commit_message>
changements de la doc et du code
changement du code pour les touchkeys et amélioration de la doc
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/pcb/bom/jeu_du_moulin_boura_Project.xlsx
+++ b/jeu_du_moulin_boura/pcb/bom/jeu_du_moulin_boura_Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/alexandre_bourquenoud_studentfr_ch/Documents/PHIE/jeu_du_moulin_alexandre_bourquenoud/jeu_du_moulin_2025_boura/jeu_du_moulin_boura/pcb/bom/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projet\jeu du moulin\jeu_du_moulin_2025_boura\jeu_du_moulin_boura\pcb\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A27B159-3A59-495E-A08E-ADA4434E27FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D028C9C-B4D1-4A56-981D-0B24940DE6D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -743,18 +743,59 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -767,12 +808,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -794,23 +829,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -827,26 +847,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1174,13 +1174,13 @@
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="28" t="str">
+      <c r="B3" s="43" t="str">
         <f>CONCATENATE("",Sheet2!A5)</f>
         <v xml:space="preserve">  1.0.0</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="45"/>
       <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="3"/>
-      <c r="I3" s="52" t="s">
+      <c r="I3" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="46"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="39"/>
     </row>
     <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
@@ -1209,46 +1209,46 @@
     </row>
     <row r="5" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="38"/>
+      <c r="C5" s="51"/>
       <c r="D5" s="5"/>
       <c r="E5" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="53" t="s">
+      <c r="F5" s="40" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="41"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="33"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
-      <c r="B6" s="26" t="str">
+      <c r="B6" s="30" t="str">
         <f>Sheet2!A4</f>
         <v>1.0.0</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="54" t="s">
+      <c r="C6" s="31"/>
+      <c r="D6" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="24"/>
+      <c r="F6" s="41"/>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="41"/>
-      <c r="L6" s="41"/>
-      <c r="M6" s="41"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="33"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
     </row>
     <row r="7" spans="1:13" ht="13.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
@@ -1256,14 +1256,14 @@
       <c r="C7" s="14"/>
       <c r="D7" s="6"/>
       <c r="E7" s="12"/>
-      <c r="F7" s="25"/>
+      <c r="F7" s="42"/>
       <c r="G7" s="11"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
@@ -1275,10 +1275,10 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="41"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="33"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
@@ -1290,10 +1290,10 @@
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
-      <c r="J9" s="41"/>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
+      <c r="M9" s="33"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="4"/>
@@ -1302,13 +1302,13 @@
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="4"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="43"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="44"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="35"/>
+      <c r="K10" s="35"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="36"/>
     </row>
     <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
@@ -1324,13 +1324,13 @@
     </row>
     <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
-      <c r="B12" s="34" t="str">
+      <c r="B12" s="47" t="str">
         <f>B3</f>
         <v xml:space="preserve">  1.0.0</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="36"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="49"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -1341,14 +1341,14 @@
       <c r="A13" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="31"/>
-      <c r="D13" s="39" t="s">
+      <c r="C13" s="46"/>
+      <c r="D13" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="40"/>
+      <c r="E13" s="53"/>
       <c r="F13" s="8" t="s">
         <v>34</v>
       </c>
@@ -1376,17 +1376,17 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="18">
-        <f>ROW(B13) - ROW($B$12)</f>
+        <f t="shared" ref="A14:A34" si="0">ROW(B13) - ROW($B$12)</f>
         <v>1</v>
       </c>
-      <c r="B14" s="33">
+      <c r="B14" s="29">
         <v>1</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="26" t="s">
+      <c r="C14" s="29"/>
+      <c r="D14" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="31"/>
       <c r="F14" s="17" t="s">
         <v>35</v>
       </c>
@@ -1401,23 +1401,23 @@
       <c r="K14" s="18"/>
       <c r="L14" s="20"/>
       <c r="M14" s="20">
-        <f>L14*B14</f>
+        <f t="shared" ref="M14:M34" si="1">L14*B14</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A15" s="18">
-        <f>ROW(B14) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="B15" s="32">
         <v>5</v>
       </c>
       <c r="C15" s="32"/>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="31"/>
       <c r="F15" s="17" t="s">
         <v>36</v>
       </c>
@@ -1432,23 +1432,23 @@
       <c r="K15" s="18"/>
       <c r="L15" s="20"/>
       <c r="M15" s="20">
-        <f>L15*B15</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="18">
-        <f>ROW(B15) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B16" s="33">
+      <c r="B16" s="29">
         <v>3</v>
       </c>
-      <c r="C16" s="33"/>
-      <c r="D16" s="26" t="s">
+      <c r="C16" s="29"/>
+      <c r="D16" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="27"/>
+      <c r="E16" s="31"/>
       <c r="F16" s="17" t="s">
         <v>37</v>
       </c>
@@ -1463,23 +1463,23 @@
       <c r="K16" s="18"/>
       <c r="L16" s="20"/>
       <c r="M16" s="20">
-        <f>L16*B16</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A17" s="18">
-        <f>ROW(B16) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B17" s="32">
         <v>4</v>
       </c>
       <c r="C17" s="32"/>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="27"/>
+      <c r="E17" s="31"/>
       <c r="F17" s="17" t="s">
         <v>38</v>
       </c>
@@ -1494,23 +1494,23 @@
       <c r="K17" s="18"/>
       <c r="L17" s="20"/>
       <c r="M17" s="20">
-        <f>L17*B17</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="90" x14ac:dyDescent="0.2">
       <c r="A18" s="18">
-        <f>ROW(B17) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="29">
         <v>24</v>
       </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="26" t="s">
+      <c r="C18" s="29"/>
+      <c r="D18" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="27"/>
+      <c r="E18" s="31"/>
       <c r="F18" s="17" t="s">
         <v>17</v>
       </c>
@@ -1533,23 +1533,23 @@
         <v>0.40200000000000002</v>
       </c>
       <c r="M18" s="20">
-        <f>L18*B18</f>
+        <f t="shared" si="1"/>
         <v>9.6479999999999997</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A19" s="18">
-        <f>ROW(B18) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B19" s="32">
         <v>1</v>
       </c>
       <c r="C19" s="32"/>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="27"/>
+      <c r="E19" s="31"/>
       <c r="F19" s="17" t="s">
         <v>39</v>
       </c>
@@ -1572,23 +1572,23 @@
         <v>9.5460000000000003E-2</v>
       </c>
       <c r="M19" s="20">
-        <f>L19*B19</f>
+        <f t="shared" si="1"/>
         <v>9.5460000000000003E-2</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A20" s="18">
-        <f>ROW(B19) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="29">
         <v>1</v>
       </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="26" t="s">
+      <c r="C20" s="29"/>
+      <c r="D20" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="27"/>
+      <c r="E20" s="31"/>
       <c r="F20" s="17" t="s">
         <v>40</v>
       </c>
@@ -1611,23 +1611,23 @@
         <v>4.62</v>
       </c>
       <c r="M20" s="20">
-        <f>L20*B20</f>
+        <f t="shared" si="1"/>
         <v>4.62</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A21" s="18">
-        <f>ROW(B20) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B21" s="32">
         <v>1</v>
       </c>
       <c r="C21" s="32"/>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="27"/>
+      <c r="E21" s="31"/>
       <c r="F21" s="17" t="s">
         <v>41</v>
       </c>
@@ -1650,23 +1650,23 @@
         <v>0.48924000000000001</v>
       </c>
       <c r="M21" s="20">
-        <f>L21*B21</f>
+        <f t="shared" si="1"/>
         <v>0.48924000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A22" s="18">
-        <f>ROW(B21) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B22" s="33">
+      <c r="B22" s="29">
         <v>1</v>
       </c>
-      <c r="C22" s="33"/>
-      <c r="D22" s="26" t="s">
+      <c r="C22" s="29"/>
+      <c r="D22" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="31"/>
       <c r="F22" s="17" t="s">
         <v>42</v>
       </c>
@@ -1689,23 +1689,23 @@
         <v>0.54</v>
       </c>
       <c r="M22" s="20">
-        <f>L22*B22</f>
+        <f t="shared" si="1"/>
         <v>0.54</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="18">
-        <f>ROW(B22) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B23" s="32">
         <v>1</v>
       </c>
       <c r="C23" s="32"/>
-      <c r="D23" s="26" t="s">
+      <c r="D23" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="31"/>
       <c r="F23" s="17" t="s">
         <v>43</v>
       </c>
@@ -1718,23 +1718,23 @@
       <c r="K23" s="18"/>
       <c r="L23" s="20"/>
       <c r="M23" s="20">
-        <f>L23*B23</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A24" s="18">
-        <f>ROW(B23) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="29">
         <v>11</v>
       </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="26" t="s">
+      <c r="C24" s="29"/>
+      <c r="D24" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="27"/>
+      <c r="E24" s="31"/>
       <c r="F24" s="17" t="s">
         <v>44</v>
       </c>
@@ -1747,23 +1747,23 @@
       <c r="K24" s="18"/>
       <c r="L24" s="20"/>
       <c r="M24" s="20">
-        <f>L24*B24</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="18">
-        <f>ROW(B24) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B25" s="32">
         <v>1</v>
       </c>
       <c r="C25" s="32"/>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="E25" s="27"/>
+      <c r="E25" s="31"/>
       <c r="F25" s="17" t="s">
         <v>45</v>
       </c>
@@ -1776,23 +1776,23 @@
       <c r="K25" s="18"/>
       <c r="L25" s="20"/>
       <c r="M25" s="20">
-        <f>L25*B25</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="18">
-        <f>ROW(B25) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B26" s="33">
+      <c r="B26" s="29">
         <v>1</v>
       </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="26" t="s">
+      <c r="C26" s="29"/>
+      <c r="D26" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="27"/>
+      <c r="E26" s="31"/>
       <c r="F26" s="17" t="s">
         <v>46</v>
       </c>
@@ -1805,23 +1805,23 @@
       <c r="K26" s="18"/>
       <c r="L26" s="20"/>
       <c r="M26" s="20">
-        <f>L26*B26</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A27" s="18">
-        <f>ROW(B26) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B27" s="32">
         <v>2</v>
       </c>
       <c r="C27" s="32"/>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="27"/>
+      <c r="E27" s="31"/>
       <c r="F27" s="17" t="s">
         <v>47</v>
       </c>
@@ -1844,23 +1844,23 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="M27" s="20">
-        <f>L27*B27</f>
+        <f t="shared" si="1"/>
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A28" s="18">
-        <f>ROW(B27) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B28" s="33">
+      <c r="B28" s="29">
         <v>11</v>
       </c>
-      <c r="C28" s="33"/>
-      <c r="D28" s="26" t="s">
+      <c r="C28" s="29"/>
+      <c r="D28" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="E28" s="27"/>
+      <c r="E28" s="31"/>
       <c r="F28" s="17" t="s">
         <v>48</v>
       </c>
@@ -1873,23 +1873,23 @@
       <c r="K28" s="18"/>
       <c r="L28" s="20"/>
       <c r="M28" s="20">
-        <f>L28*B28</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="18">
-        <f>ROW(B28) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B29" s="32">
         <v>1</v>
       </c>
       <c r="C29" s="32"/>
-      <c r="D29" s="26" t="s">
+      <c r="D29" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="E29" s="27"/>
+      <c r="E29" s="31"/>
       <c r="F29" s="17" t="s">
         <v>49</v>
       </c>
@@ -1912,23 +1912,23 @@
         <v>0.75</v>
       </c>
       <c r="M29" s="20">
-        <f>L29*B29</f>
+        <f t="shared" si="1"/>
         <v>0.75</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="18">
-        <f>ROW(B29) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="29">
         <v>2</v>
       </c>
-      <c r="C30" s="33"/>
-      <c r="D30" s="26" t="s">
+      <c r="C30" s="29"/>
+      <c r="D30" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="31"/>
       <c r="F30" s="17" t="s">
         <v>50</v>
       </c>
@@ -1951,23 +1951,23 @@
         <v>0.39</v>
       </c>
       <c r="M30" s="20">
-        <f>L30*B30</f>
+        <f t="shared" si="1"/>
         <v>0.78</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="18">
-        <f>ROW(B30) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B31" s="32">
         <v>2</v>
       </c>
       <c r="C31" s="32"/>
-      <c r="D31" s="26" t="s">
+      <c r="D31" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E31" s="27"/>
+      <c r="E31" s="31"/>
       <c r="F31" s="17" t="s">
         <v>51</v>
       </c>
@@ -1990,23 +1990,23 @@
         <v>0.39</v>
       </c>
       <c r="M31" s="20">
-        <f>L31*B31</f>
+        <f t="shared" si="1"/>
         <v>0.78</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A32" s="18">
-        <f>ROW(B31) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B32" s="33">
+      <c r="B32" s="29">
         <v>4</v>
       </c>
-      <c r="C32" s="33"/>
-      <c r="D32" s="26" t="s">
+      <c r="C32" s="29"/>
+      <c r="D32" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="E32" s="27"/>
+      <c r="E32" s="31"/>
       <c r="F32" s="17" t="s">
         <v>52</v>
       </c>
@@ -2019,23 +2019,23 @@
       <c r="K32" s="18"/>
       <c r="L32" s="20"/>
       <c r="M32" s="20">
-        <f>L32*B32</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="18">
-        <f>ROW(B32) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B33" s="32">
         <v>1</v>
       </c>
       <c r="C33" s="32"/>
-      <c r="D33" s="26" t="s">
+      <c r="D33" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E33" s="27"/>
+      <c r="E33" s="31"/>
       <c r="F33" s="17" t="s">
         <v>53</v>
       </c>
@@ -2048,23 +2048,23 @@
       <c r="K33" s="18"/>
       <c r="L33" s="20"/>
       <c r="M33" s="20">
-        <f>L33*B33</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A34" s="18">
-        <f>ROW(B33) - ROW($B$12)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B34" s="33">
+      <c r="B34" s="29">
         <v>1</v>
       </c>
-      <c r="C34" s="33"/>
-      <c r="D34" s="26" t="s">
+      <c r="C34" s="29"/>
+      <c r="D34" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="E34" s="27"/>
+      <c r="E34" s="31"/>
       <c r="F34" s="17" t="s">
         <v>54</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>0.7</v>
       </c>
       <c r="M34" s="20">
-        <f>L34*B34</f>
+        <f t="shared" si="1"/>
         <v>0.7</v>
       </c>
     </row>
@@ -2108,51 +2108,6 @@
     <row r="37" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="G10:M10"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="J7:M7"/>
     <mergeCell ref="F5:F7"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="B3:E3"/>
@@ -2164,6 +2119,51 @@
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D13:E13"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="G10:M10"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="D33:E33"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2183,21 +2183,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="54" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="48"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="56"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="26" t="s">
         <v>115</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="26" t="s">
         <v>116</v>
       </c>
       <c r="B3" s="1"/>
@@ -2220,17 +2220,17 @@
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="27" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="28" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="26" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2242,13 +2242,13 @@
     </row>
     <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:4" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="49" t="e">
+      <c r="A13" s="57" t="e">
         <f>CONCATENATE(Sheet2!A18,"[",Sheet2!#REF!,"]",Sheet2!#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="51"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
@@ -2272,15 +2272,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010098AFC7C83C7C054E95F4B42F91168742" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="66e3d8284d9fc5410f6939df54f0caa6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c73ba516-6d34-4b92-a096-ac7dfb020022" xmlns:ns3="ebd706b7-678b-40df-972d-f0eaa6262b36" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ea909251fc86ece970dc0ed8cbb70340" ns2:_="" ns3:_="">
     <xsd:import namespace="c73ba516-6d34-4b92-a096-ac7dfb020022"/>
@@ -2487,15 +2478,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C64E99E-77F3-4A44-9FA2-482228DEF9ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCF1807D-2C11-4442-B446-3E1610E4AAB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2512,4 +2504,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C64E99E-77F3-4A44-9FA2-482228DEF9ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changements dans la doc et dans le code
Ajout de beaucoup d'élements dans la documentation et changement du fonctionnement du code pour essayer de faire fonctionner les touches capacitives
</commit_message>
<xml_diff>
--- a/jeu_du_moulin_boura/pcb/bom/jeu_du_moulin_boura_Project.xlsx
+++ b/jeu_du_moulin_boura/pcb/bom/jeu_du_moulin_boura_Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projet\jeu du moulin\jeu_du_moulin_2025_boura\jeu_du_moulin_boura\pcb\bom\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/alexandre_bourquenoud_studentfr_ch/Documents/PHIE/jeu_du_moulin_alexandre_bourquenoud/jeu_du_moulin_2025_boura/jeu_du_moulin_boura/pcb/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D028C9C-B4D1-4A56-981D-0B24940DE6D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9D028C9C-B4D1-4A56-981D-0B24940DE6D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0958805C-4E0A-473D-91D0-90A51744297D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="117">
   <si>
     <t>Désignation:</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t>Zener 2.4V</t>
-  </si>
-  <si>
-    <t>STM32L072CZT6</t>
   </si>
   <si>
     <t>Voltage Regulator 3.3V</t>
@@ -754,16 +751,58 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -786,48 +825,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1174,13 +1171,13 @@
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="43" t="str">
+      <c r="B3" s="34" t="str">
         <f>CONCATENATE("",Sheet2!A5)</f>
         <v xml:space="preserve">  1.0.0</v>
       </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="45"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="36"/>
       <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
@@ -1188,13 +1185,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="3"/>
-      <c r="I3" s="37" t="s">
+      <c r="I3" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="39"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="53"/>
     </row>
     <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
@@ -1209,46 +1206,46 @@
     </row>
     <row r="5" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="51"/>
+      <c r="C5" s="44"/>
       <c r="D5" s="5"/>
       <c r="E5" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="29" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
+      <c r="J5" s="47"/>
+      <c r="K5" s="47"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
-      <c r="B6" s="30" t="str">
+      <c r="B6" s="32" t="str">
         <f>Sheet2!A4</f>
         <v>1.0.0</v>
       </c>
-      <c r="C6" s="31"/>
+      <c r="C6" s="33"/>
       <c r="D6" s="24" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="41"/>
+      <c r="F6" s="30"/>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="33"/>
-      <c r="L6" s="33"/>
-      <c r="M6" s="33"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="47"/>
     </row>
     <row r="7" spans="1:13" ht="13.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
@@ -1256,14 +1253,14 @@
       <c r="C7" s="14"/>
       <c r="D7" s="6"/>
       <c r="E7" s="12"/>
-      <c r="F7" s="42"/>
+      <c r="F7" s="31"/>
       <c r="G7" s="11"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
@@ -1275,10 +1272,10 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="33"/>
-      <c r="M8" s="33"/>
+      <c r="J8" s="47"/>
+      <c r="K8" s="47"/>
+      <c r="L8" s="47"/>
+      <c r="M8" s="47"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
@@ -1290,10 +1287,10 @@
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="33"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="47"/>
+      <c r="L9" s="47"/>
+      <c r="M9" s="47"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="4"/>
@@ -1302,13 +1299,13 @@
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="4"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="35"/>
-      <c r="L10" s="35"/>
-      <c r="M10" s="36"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="50"/>
     </row>
     <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
@@ -1324,13 +1321,13 @@
     </row>
     <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
-      <c r="B12" s="47" t="str">
+      <c r="B12" s="40" t="str">
         <f>B3</f>
         <v xml:space="preserve">  1.0.0</v>
       </c>
-      <c r="C12" s="48"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="49"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="42"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -1341,34 +1338,34 @@
       <c r="A13" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="46"/>
-      <c r="D13" s="52" t="s">
+      <c r="C13" s="37"/>
+      <c r="D13" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="53"/>
+      <c r="E13" s="46"/>
       <c r="F13" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M13" s="8" t="s">
         <v>6</v>
@@ -1379,23 +1376,23 @@
         <f t="shared" ref="A14:A34" si="0">ROW(B13) - ROW($B$12)</f>
         <v>1</v>
       </c>
-      <c r="B14" s="29">
+      <c r="B14" s="39">
         <v>1</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="30" t="s">
+      <c r="C14" s="39"/>
+      <c r="D14" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="31"/>
+      <c r="E14" s="33"/>
       <c r="F14" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H14" s="18"/>
       <c r="I14" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J14" s="18"/>
       <c r="K14" s="18"/>
@@ -1410,23 +1407,23 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="38">
         <v>5</v>
       </c>
-      <c r="C15" s="32"/>
-      <c r="D15" s="30" t="s">
+      <c r="C15" s="38"/>
+      <c r="D15" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="31"/>
+      <c r="E15" s="33"/>
       <c r="F15" s="17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H15" s="18"/>
       <c r="I15" s="18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
@@ -1441,23 +1438,23 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B16" s="29">
+      <c r="B16" s="39">
         <v>3</v>
       </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="30" t="s">
+      <c r="C16" s="39"/>
+      <c r="D16" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="31"/>
+      <c r="E16" s="33"/>
       <c r="F16" s="17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H16" s="18"/>
       <c r="I16" s="18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J16" s="18"/>
       <c r="K16" s="18"/>
@@ -1472,23 +1469,23 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="38">
         <v>4</v>
       </c>
-      <c r="C17" s="32"/>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="38"/>
+      <c r="D17" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="31"/>
+      <c r="E17" s="33"/>
       <c r="F17" s="17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H17" s="18"/>
       <c r="I17" s="18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J17" s="18"/>
       <c r="K17" s="18"/>
@@ -1503,31 +1500,31 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B18" s="29">
+      <c r="B18" s="39">
         <v>24</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="39"/>
+      <c r="D18" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="31"/>
+      <c r="E18" s="33"/>
       <c r="F18" s="17" t="s">
         <v>17</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I18" s="18" t="s">
         <v>17</v>
       </c>
       <c r="J18" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K18" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L18" s="20">
         <v>0.40200000000000002</v>
@@ -1542,31 +1539,31 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="38">
         <v>1</v>
       </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="30" t="s">
+      <c r="C19" s="38"/>
+      <c r="D19" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="31"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I19" s="18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J19" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K19" s="18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L19" s="20">
         <v>9.5460000000000003E-2</v>
@@ -1581,31 +1578,31 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B20" s="29">
+      <c r="B20" s="39">
         <v>1</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="31"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" s="33"/>
       <c r="F20" s="17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I20" s="18" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J20" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L20" s="20">
         <v>4.62</v>
@@ -1620,31 +1617,31 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B21" s="32">
+      <c r="B21" s="38">
         <v>1</v>
       </c>
-      <c r="C21" s="32"/>
-      <c r="D21" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="31"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="33"/>
       <c r="F21" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I21" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J21" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K21" s="18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L21" s="20">
         <v>0.48924000000000001</v>
@@ -1659,31 +1656,31 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B22" s="29">
+      <c r="B22" s="39">
         <v>1</v>
       </c>
-      <c r="C22" s="29"/>
-      <c r="D22" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="E22" s="31"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="33"/>
       <c r="F22" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I22" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J22" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K22" s="18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L22" s="20">
         <v>0.54</v>
@@ -1698,19 +1695,19 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B23" s="32">
+      <c r="B23" s="38">
         <v>1</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="31"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="33"/>
       <c r="F23" s="17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G23" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H23" s="18"/>
       <c r="I23" s="18"/>
@@ -1727,19 +1724,19 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="39">
         <v>11</v>
       </c>
-      <c r="C24" s="29"/>
-      <c r="D24" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="31"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="33"/>
       <c r="F24" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H24" s="18"/>
       <c r="I24" s="18"/>
@@ -1756,19 +1753,19 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="38">
         <v>1</v>
       </c>
-      <c r="C25" s="32"/>
-      <c r="D25" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="E25" s="31"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="E25" s="33"/>
       <c r="F25" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G25" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H25" s="18"/>
       <c r="I25" s="18"/>
@@ -1785,19 +1782,19 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B26" s="29">
+      <c r="B26" s="39">
         <v>1</v>
       </c>
-      <c r="C26" s="29"/>
-      <c r="D26" s="30" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="31"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="33"/>
       <c r="F26" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G26" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H26" s="18"/>
       <c r="I26" s="18"/>
@@ -1814,31 +1811,31 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="38">
         <v>2</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="E27" s="31"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="33"/>
       <c r="F27" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G27" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I27" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J27" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K27" s="18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L27" s="20">
         <v>8.9999999999999993E-3</v>
@@ -1853,19 +1850,19 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B28" s="29">
+      <c r="B28" s="39">
         <v>11</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="E28" s="31"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="33"/>
       <c r="F28" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
@@ -1882,31 +1879,31 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B29" s="32">
+      <c r="B29" s="38">
         <v>1</v>
       </c>
-      <c r="C29" s="32"/>
-      <c r="D29" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="E29" s="31"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="33"/>
       <c r="F29" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I29" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J29" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K29" s="18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L29" s="20">
         <v>0.75</v>
@@ -1921,31 +1918,31 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B30" s="29">
+      <c r="B30" s="39">
         <v>2</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="31"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="33"/>
       <c r="F30" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I30" s="18">
         <v>5000</v>
       </c>
       <c r="J30" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L30" s="20">
         <v>0.39</v>
@@ -1960,31 +1957,31 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B31" s="32">
+      <c r="B31" s="38">
         <v>2</v>
       </c>
-      <c r="C31" s="32"/>
-      <c r="D31" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="E31" s="31"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E31" s="33"/>
       <c r="F31" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I31" s="18">
         <v>5001</v>
       </c>
       <c r="J31" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K31" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L31" s="20">
         <v>0.39</v>
@@ -1999,19 +1996,19 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B32" s="29">
+      <c r="B32" s="39">
         <v>4</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="E32" s="31"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E32" s="33"/>
       <c r="F32" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
@@ -2028,19 +2025,19 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B33" s="32">
+      <c r="B33" s="38">
         <v>1</v>
       </c>
-      <c r="C33" s="32"/>
-      <c r="D33" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="E33" s="31"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="E33" s="33"/>
       <c r="F33" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H33" s="18"/>
       <c r="I33" s="18"/>
@@ -2057,31 +2054,31 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="39">
         <v>1</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="E34" s="31"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="E34" s="33"/>
       <c r="F34" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I34" s="18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J34" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K34" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L34" s="20">
         <v>0.7</v>
@@ -2108,6 +2105,51 @@
     <row r="37" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="56">
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="G10:M10"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="J7:M7"/>
     <mergeCell ref="F5:F7"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="B3:E3"/>
@@ -2119,51 +2161,6 @@
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D13:E13"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="G10:M10"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:E33"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2184,21 +2181,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="54" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="56"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -2221,7 +2218,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2231,7 +2228,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -2272,6 +2269,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010098AFC7C83C7C054E95F4B42F91168742" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="66e3d8284d9fc5410f6939df54f0caa6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c73ba516-6d34-4b92-a096-ac7dfb020022" xmlns:ns3="ebd706b7-678b-40df-972d-f0eaa6262b36" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ea909251fc86ece970dc0ed8cbb70340" ns2:_="" ns3:_="">
     <xsd:import namespace="c73ba516-6d34-4b92-a096-ac7dfb020022"/>
@@ -2478,16 +2484,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C64E99E-77F3-4A44-9FA2-482228DEF9ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCF1807D-2C11-4442-B446-3E1610E4AAB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2504,12 +2509,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C64E99E-77F3-4A44-9FA2-482228DEF9ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>